<commit_message>
instructor resources filled out
</commit_message>
<xml_diff>
--- a/courses/Reg/DailyRecord.xlsx
+++ b/courses/Reg/DailyRecord.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hbarreto\Documents\GitHub\homepage\courses\Reg\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{016C9230-D97C-4A77-A810-C52738AFC992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EA7373B-C5AB-4875-8D2B-570DDA67DF0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="257">
   <si>
     <t>Grade</t>
   </si>
@@ -132,9 +132,6 @@
     <t>Multivariate Regression Workshop</t>
   </si>
   <si>
-    <t>FALL BREAK</t>
-  </si>
-  <si>
     <t>Confidence Intervals</t>
   </si>
   <si>
@@ -151,9 +148,6 @@
   </si>
   <si>
     <t>i.firmsize</t>
-  </si>
-  <si>
-    <t>Complex Surveys and Unequal Probability of Selection</t>
   </si>
   <si>
     <r>
@@ -220,9 +214,6 @@
   </si>
   <si>
     <t>Heteroskedasticity: GLS</t>
-  </si>
-  <si>
-    <t>BUS 305: Regression with Microdata</t>
   </si>
   <si>
     <t>Syllabus, Basic stats on INCWAGE, avg is min SSR</t>
@@ -480,9 +471,6 @@
     <t>Reg results table</t>
   </si>
   <si>
-    <t>33.pdf</t>
-  </si>
-  <si>
     <t>Use SAMPLE, sim</t>
   </si>
   <si>
@@ -490,15 +478,6 @@
   </si>
   <si>
     <t>Study</t>
-  </si>
-  <si>
-    <t>Orthoreg.xlsm</t>
-  </si>
-  <si>
-    <t>EqualUnequalProb.xlsm</t>
-  </si>
-  <si>
-    <t>Matriculation.xlsx</t>
   </si>
   <si>
     <t>In Excel file</t>
@@ -553,138 +532,6 @@
     <t>Passcode: E+a46@yb</t>
   </si>
   <si>
-    <t>Song</t>
-  </si>
-  <si>
-    <t>Pitbull Guantanamera</t>
-  </si>
-  <si>
-    <t>Irakere Marie Laveaux</t>
-  </si>
-  <si>
-    <t>Viene a pedir mi mano</t>
-  </si>
-  <si>
-    <t>Chan Chan</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=tGbRZ73NvlY</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=o5cELP06Mik&amp;t=2s</t>
-  </si>
-  <si>
-    <t>Telephone Line</t>
-  </si>
-  <si>
-    <t>El Cuarto de Tula video</t>
-  </si>
-  <si>
-    <t>One tin soldier video</t>
-  </si>
-  <si>
-    <t>Let's Stay Together</t>
-  </si>
-  <si>
-    <t>Mi Tierra</t>
-  </si>
-  <si>
-    <t>This Land is Your Land</t>
-  </si>
-  <si>
-    <t>Cuban Elvis</t>
-  </si>
-  <si>
-    <t>Guantanamera</t>
-  </si>
-  <si>
-    <t>Ojala que llueva café</t>
-  </si>
-  <si>
-    <t>Body Electric</t>
-  </si>
-  <si>
-    <t>Picabo Street skiing video</t>
-  </si>
-  <si>
-    <t>rocky raccoon</t>
-  </si>
-  <si>
-    <t>Fire on High</t>
-  </si>
-  <si>
-    <t>City of New Orleans</t>
-  </si>
-  <si>
-    <t>Heart of Gold</t>
-  </si>
-  <si>
-    <t>Band of Gold</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=jhuDgUnqXUY&amp;t=16s</t>
-  </si>
-  <si>
-    <t>Lido Shuffle</t>
-  </si>
-  <si>
-    <t>Marvin</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=FrkEDe6Ljqs</t>
-  </si>
-  <si>
-    <t>Black or White</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=F2AitTPI5U0</t>
-  </si>
-  <si>
-    <t>Ode to Joy</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=kbJcQYVtZMo&amp;t=2s</t>
-  </si>
-  <si>
-    <t>Oye Como Va</t>
-  </si>
-  <si>
-    <t>Light My Fire</t>
-  </si>
-  <si>
-    <t>Get Ready</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=A3Ix4hKSnxQ</t>
-  </si>
-  <si>
-    <t>Everyday People</t>
-  </si>
-  <si>
-    <t>Fast Car Grammys</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=pLfH9HSUyf4</t>
-  </si>
-  <si>
-    <t>Texas Hold Em</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=ycwtqqhV6UE</t>
-  </si>
-  <si>
-    <t>Shaft</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=ZVj8FgMMAK8&amp;t=96s</t>
-  </si>
-  <si>
-    <t>Long and Winding Road</t>
-  </si>
-  <si>
-    <t>Southern Cross</t>
-  </si>
-  <si>
     <t>1.JourneyBegins</t>
   </si>
   <si>
@@ -725,9 +572,6 @@
   </si>
   <si>
     <t>1.CPSIncEducPreClass.xlsx</t>
-  </si>
-  <si>
-    <t>Every day has student and teacher Word doc</t>
   </si>
   <si>
     <t>Class Prep Notes</t>
@@ -770,9 +614,6 @@
     <t>https://depauw-edu.zoom.us/rec/share/8Ma03tb3qOC9X03KZ17FYqKAz42Jq1JklNBBzrMbhC7IZA-CA5irvVA6kClhJBkc.L4L-5dPo2Fzoaj0C</t>
   </si>
   <si>
-    <t>La Bamba</t>
-  </si>
-  <si>
     <t>Discuss OVB, Add Exp and Exp^2</t>
   </si>
   <si>
@@ -818,12 +659,6 @@
     <t>15.Measurement Error</t>
   </si>
   <si>
-    <t>Night Fever video</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=e6GB04zeDeQ</t>
-  </si>
-  <si>
     <t>Passcode: 3K5y!N+J</t>
   </si>
   <si>
@@ -848,12 +683,6 @@
     <t>https://depauw-edu.zoom.us/rec/share/0QFyjU17rgqnlj5vOEt17WY-MUKPq4s-RjiO1LflEFJPqIsVG0Q7UjRRUMXeDj6Q.Uks4lVawUOXYbB-a</t>
   </si>
   <si>
-    <t>zoom</t>
-  </si>
-  <si>
-    <t>exam</t>
-  </si>
-  <si>
     <t>Use a student's file (or 17.PreClass), save as to public folder</t>
   </si>
   <si>
@@ -905,9 +734,6 @@
     <t>https://depauw-edu.zoom.us/rec/share/uxfne8g5W8Iz48l9w14vDzOOknTC_9UrMp2YGeC16WwmrqScIE1mwLzQ-d1nPz3V.WlxMe0_ginZ5YeQy</t>
   </si>
   <si>
-    <t>air media would not play it after I adjusted the volume</t>
-  </si>
-  <si>
     <t>22 all of it</t>
   </si>
   <si>
@@ -923,9 +749,6 @@
     <t>Use 23.SEPreClass</t>
   </si>
   <si>
-    <t>Kodachrome</t>
-  </si>
-  <si>
     <t>68% CI with n=5 and n=100, understand Est SE and t dist</t>
   </si>
   <si>
@@ -957,9 +780,6 @@
   </si>
   <si>
     <t>Passcode: r%k2Fr!*</t>
-  </si>
-  <si>
-    <t>Il Paradisi</t>
   </si>
   <si>
     <t>Use 27.HetPreClass</t>
@@ -1034,6 +854,63 @@
   </si>
   <si>
     <t>Passcode: 2+ypYvp8</t>
+  </si>
+  <si>
+    <t>https://depauw-edu.zoom.us/rec/share/e_tnBj9TPBpDpJwk-M58NZFEMtq_gGstEBvRMubEQ2hXFlTkV2Ews-c_58hF0N3j.YViq6NRYyDEZQgFR</t>
+  </si>
+  <si>
+    <t>Passcode: Jdq%n7Cx</t>
+  </si>
+  <si>
+    <t>30.Partial Xs</t>
+  </si>
+  <si>
+    <t>36.Matriculation.xlsx</t>
+  </si>
+  <si>
+    <t>37.EqualUnequalProb.xlsm</t>
+  </si>
+  <si>
+    <t>https://depauw-edu.zoom.us/rec/share/LrwL07QRW0DCiQMSJT5SRdssv4ErCniVigzjECF2d8M_D4SxtHmUtl2R5s4jG2gv.DNPgpryXz8k_cGg6</t>
+  </si>
+  <si>
+    <t>Passcode: bd1^b8dU</t>
+  </si>
+  <si>
+    <t>35.Orthoreg.xlsm</t>
+  </si>
+  <si>
+    <t>https://depauw-edu.zoom.us/rec/share/IwJ29UkeOmKYMlhZXAEuajxRM2L7c2IIz4sQtigcf2x0ClN6gcy1j0GZUYMkb3gu.MH7NP4YOVcxQZjqy</t>
+  </si>
+  <si>
+    <t>Passcode: g55@@DW3</t>
+  </si>
+  <si>
+    <t>https://depauw-edu.zoom.us/rec/share/yfj8mnMWkXOUWwFr4LfZTgwOGDhNics2MNMR6Hd_8nLPcwC7_X2tFP7vLIBNsp7X.33YPJqqqXbJVfQRM</t>
+  </si>
+  <si>
+    <t>Passcode: pp@1HK.k</t>
+  </si>
+  <si>
+    <t>SPRING BREAK</t>
+  </si>
+  <si>
+    <t>Unequal Probability of Selection and WLS</t>
+  </si>
+  <si>
+    <t>BUSA 305: Regression with Microdata</t>
+  </si>
+  <si>
+    <t>Most classes have a student Word doc handout (see Google drive folder)</t>
+  </si>
+  <si>
+    <t>SPRING 2026 VERSION</t>
+  </si>
+  <si>
+    <t>Print A1:D48 for last day</t>
+  </si>
+  <si>
+    <t>copy/paste just the passcode itself</t>
   </si>
 </sst>
 </file>
@@ -1630,7 +1507,7 @@
   <sheetPr codeName="Sheet3">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R60"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr defaultRowHeight="11.4"/>
   <cols>
     <col min="3" max="3" width="8.625" customWidth="1"/>
@@ -1638,35 +1515,39 @@
     <col min="5" max="5" width="59" customWidth="1"/>
     <col min="6" max="6" width="27" customWidth="1"/>
     <col min="7" max="7" width="27.75" customWidth="1"/>
-    <col min="8" max="8" width="58.75" customWidth="1"/>
-    <col min="9" max="9" width="11.75" customWidth="1"/>
+    <col min="8" max="8" width="62.875" customWidth="1"/>
+    <col min="9" max="9" width="24.625" customWidth="1"/>
+    <col min="10" max="10" width="21.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="17.399999999999999">
+    <row r="1" spans="1:11" ht="17.399999999999999">
       <c r="A1" s="11" t="s">
-        <v>49</v>
+        <v>252</v>
       </c>
       <c r="C1" s="4"/>
       <c r="D1" s="5"/>
-    </row>
-    <row r="2" spans="1:18" ht="13.2">
+      <c r="E1" s="1" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="13.2">
       <c r="A2" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="4"/>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:11">
       <c r="A3" s="24" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="C3" s="1"/>
       <c r="H3" s="1" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" ht="16.2" thickBot="1">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="16.2" thickBot="1">
       <c r="A4" s="12" t="s">
         <v>6</v>
       </c>
@@ -1683,23 +1564,20 @@
         <v>12</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>286</v>
+        <v>226</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="H4" s="22" t="s">
-        <v>203</v>
+        <v>151</v>
       </c>
       <c r="I4" s="28" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="J4" s="28"/>
-      <c r="L4" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="15.6">
+    </row>
+    <row r="5" spans="1:11" ht="15.6">
       <c r="A5" s="2">
         <v>46048</v>
       </c>
@@ -1711,31 +1589,31 @@
         <v>Mon</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F5" t="s">
-        <v>188</v>
+        <v>137</v>
       </c>
       <c r="G5" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="H5" t="s">
-        <v>201</v>
+        <v>150</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="J5" t="s">
-        <v>143</v>
-      </c>
-      <c r="L5" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" ht="15.6">
+        <v>136</v>
+      </c>
+      <c r="K5" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="15.6">
       <c r="A6" s="2">
         <f>A5+2</f>
         <v>46050</v>
@@ -1754,25 +1632,22 @@
         <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>189</v>
+        <v>138</v>
       </c>
       <c r="G6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="H6" t="s">
-        <v>190</v>
+        <v>139</v>
       </c>
       <c r="I6" s="24" t="s">
-        <v>191</v>
+        <v>140</v>
       </c>
       <c r="J6" t="s">
-        <v>192</v>
-      </c>
-      <c r="L6" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" ht="24">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="24">
       <c r="A7" s="2">
         <f>A6+2</f>
         <v>46052</v>
@@ -1791,25 +1666,22 @@
         <v>16</v>
       </c>
       <c r="F7" t="s">
-        <v>193</v>
+        <v>142</v>
       </c>
       <c r="G7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="H7" s="26" t="s">
-        <v>204</v>
+        <v>152</v>
       </c>
       <c r="I7" s="24" t="s">
-        <v>195</v>
+        <v>144</v>
       </c>
       <c r="J7" t="s">
-        <v>194</v>
-      </c>
-      <c r="L7" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" ht="15.6">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="15.6">
       <c r="A8" s="2">
         <f>A5+7</f>
         <v>46055</v>
@@ -1828,25 +1700,22 @@
         <v>18</v>
       </c>
       <c r="F8" t="s">
-        <v>198</v>
+        <v>147</v>
       </c>
       <c r="G8" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="H8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="I8" s="24" t="s">
-        <v>196</v>
+        <v>145</v>
       </c>
       <c r="J8" t="s">
-        <v>197</v>
-      </c>
-      <c r="L8" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="15.6">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="15.6">
       <c r="A9" s="2">
         <f t="shared" ref="A9:A15" si="1">A6+7</f>
         <v>46057</v>
@@ -1865,31 +1734,22 @@
         <v>20</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G9" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="I9" s="24" t="s">
-        <v>200</v>
+        <v>149</v>
       </c>
       <c r="J9" t="s">
-        <v>199</v>
-      </c>
-      <c r="L9" t="s">
         <v>148</v>
       </c>
-      <c r="M9" s="24" t="s">
-        <v>149</v>
-      </c>
-      <c r="R9" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="15.6">
+    </row>
+    <row r="10" spans="1:11" ht="15.6">
       <c r="A10" s="2">
         <f t="shared" si="1"/>
         <v>46059</v>
@@ -1902,34 +1762,28 @@
         <v>Fri</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="E10" t="s">
-        <v>206</v>
+        <v>154</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G10" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="H10" t="s">
-        <v>205</v>
+        <v>153</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>208</v>
+        <v>156</v>
       </c>
       <c r="J10" t="s">
-        <v>207</v>
-      </c>
-      <c r="L10" t="s">
-        <v>180</v>
-      </c>
-      <c r="M10" s="24" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" ht="15.6">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="15.6">
       <c r="A11" s="2">
         <f t="shared" si="1"/>
         <v>46062</v>
@@ -1942,31 +1796,28 @@
         <v>Mon</v>
       </c>
       <c r="D11" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" t="s">
         <v>61</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="F11" t="s">
-        <v>63</v>
-      </c>
-      <c r="G11" t="s">
-        <v>64</v>
-      </c>
       <c r="H11" t="s">
-        <v>212</v>
+        <v>160</v>
       </c>
       <c r="I11" s="24" t="s">
-        <v>210</v>
+        <v>158</v>
       </c>
       <c r="J11" t="s">
-        <v>209</v>
-      </c>
-      <c r="L11" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="15.6">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="15.6">
       <c r="A12" s="2">
         <f t="shared" si="1"/>
         <v>46064</v>
@@ -1979,31 +1830,28 @@
         <v>Wed</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E12" t="s">
-        <v>217</v>
+        <v>164</v>
       </c>
       <c r="F12" t="s">
-        <v>211</v>
+        <v>159</v>
       </c>
       <c r="G12" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="H12" t="s">
-        <v>213</v>
+        <v>161</v>
       </c>
       <c r="I12" s="24" t="s">
-        <v>215</v>
+        <v>163</v>
       </c>
       <c r="J12" t="s">
-        <v>214</v>
-      </c>
-      <c r="L12" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="15.6">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="15.6">
       <c r="A13" s="2">
         <f t="shared" si="1"/>
         <v>46066</v>
@@ -2016,31 +1864,28 @@
         <v>Fri</v>
       </c>
       <c r="D13" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E13" t="s">
+        <v>165</v>
+      </c>
+      <c r="F13" t="s">
+        <v>65</v>
+      </c>
+      <c r="G13" t="s">
+        <v>66</v>
+      </c>
+      <c r="H13" t="s">
         <v>67</v>
       </c>
-      <c r="E13" t="s">
-        <v>218</v>
-      </c>
-      <c r="F13" t="s">
-        <v>68</v>
-      </c>
-      <c r="G13" t="s">
-        <v>69</v>
-      </c>
-      <c r="H13" t="s">
-        <v>70</v>
-      </c>
       <c r="I13" s="24" t="s">
-        <v>220</v>
+        <v>167</v>
       </c>
       <c r="J13" t="s">
-        <v>219</v>
-      </c>
-      <c r="L13" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" ht="15.6">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="15.6">
       <c r="A14" s="2">
         <f t="shared" si="1"/>
         <v>46069</v>
@@ -2056,28 +1901,25 @@
         <v>21</v>
       </c>
       <c r="E14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" t="s">
+        <v>69</v>
+      </c>
+      <c r="G14" t="s">
+        <v>70</v>
+      </c>
+      <c r="H14" t="s">
         <v>71</v>
       </c>
-      <c r="F14" t="s">
-        <v>72</v>
-      </c>
-      <c r="G14" t="s">
-        <v>73</v>
-      </c>
-      <c r="H14" t="s">
-        <v>74</v>
-      </c>
       <c r="I14" s="24" t="s">
-        <v>222</v>
+        <v>169</v>
       </c>
       <c r="J14" t="s">
-        <v>221</v>
-      </c>
-      <c r="L14" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" ht="15.6">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="15.6">
       <c r="A15" s="2">
         <f t="shared" si="1"/>
         <v>46071</v>
@@ -2090,31 +1932,28 @@
         <v>Wed</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E15" t="s">
         <v>22</v>
       </c>
       <c r="F15" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="H15" t="s">
-        <v>223</v>
+        <v>170</v>
       </c>
       <c r="I15" s="24" t="s">
-        <v>225</v>
+        <v>172</v>
       </c>
       <c r="J15" t="s">
-        <v>224</v>
-      </c>
-      <c r="L15" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" ht="15.6">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="15.6">
       <c r="A16" s="2">
         <f>A15+2</f>
         <v>46073</v>
@@ -2133,25 +1972,22 @@
         <v>24</v>
       </c>
       <c r="F16" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G16" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="H16" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>227</v>
+        <v>174</v>
       </c>
       <c r="J16" t="s">
-        <v>226</v>
-      </c>
-      <c r="L16" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="15.6">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="15.6">
       <c r="A17" s="2">
         <f>A16+3</f>
         <v>46076</v>
@@ -2164,28 +2000,25 @@
         <v>Mon</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E17" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F17" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="G17" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>229</v>
+        <v>176</v>
       </c>
       <c r="J17" t="s">
-        <v>228</v>
-      </c>
-      <c r="L17" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="15.6">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="15.6">
       <c r="A18" s="2">
         <f>A17+2</f>
         <v>46078</v>
@@ -2201,14 +2034,11 @@
         <v>1</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>230</v>
+        <v>177</v>
       </c>
       <c r="G18" s="6"/>
-      <c r="L18" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="15.6">
+    </row>
+    <row r="19" spans="1:10" ht="15.6">
       <c r="A19" s="2">
         <f>A18+2</f>
         <v>46080</v>
@@ -2221,34 +2051,28 @@
         <v>Fri</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E19" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F19" t="s">
-        <v>231</v>
+        <v>178</v>
       </c>
       <c r="G19" t="s">
-        <v>237</v>
+        <v>182</v>
       </c>
       <c r="H19" t="s">
-        <v>236</v>
+        <v>181</v>
       </c>
       <c r="I19" s="24" t="s">
-        <v>235</v>
+        <v>180</v>
       </c>
       <c r="J19" t="s">
-        <v>234</v>
-      </c>
-      <c r="L19" t="s">
-        <v>232</v>
-      </c>
-      <c r="M19" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" ht="15.6">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="15.6">
       <c r="A20" s="2">
         <f>A17+7</f>
         <v>46083</v>
@@ -2264,28 +2088,25 @@
         <v>25</v>
       </c>
       <c r="E20" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="F20" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="G20" t="s">
-        <v>238</v>
+        <v>183</v>
       </c>
       <c r="H20" t="s">
-        <v>239</v>
+        <v>184</v>
       </c>
       <c r="I20" s="24" t="s">
-        <v>241</v>
+        <v>186</v>
       </c>
       <c r="J20" t="s">
-        <v>240</v>
-      </c>
-      <c r="L20" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" ht="15.6">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="15.6">
       <c r="A21" s="2">
         <f>A18+7</f>
         <v>46085</v>
@@ -2298,31 +2119,28 @@
         <v>Wed</v>
       </c>
       <c r="D21" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="E21" t="s">
+        <v>86</v>
+      </c>
+      <c r="F21" t="s">
+        <v>87</v>
+      </c>
+      <c r="G21" t="s">
         <v>88</v>
       </c>
-      <c r="E21" t="s">
-        <v>89</v>
-      </c>
-      <c r="F21" t="s">
-        <v>90</v>
-      </c>
-      <c r="G21" t="s">
-        <v>91</v>
-      </c>
       <c r="H21" t="s">
-        <v>244</v>
+        <v>187</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>246</v>
+        <v>189</v>
       </c>
       <c r="J21" t="s">
-        <v>245</v>
-      </c>
-      <c r="L21" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" ht="15.6">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="15.6">
       <c r="A22" s="2">
         <f>A21+2</f>
         <v>46087</v>
@@ -2338,28 +2156,25 @@
         <v>26</v>
       </c>
       <c r="E22" t="s">
+        <v>89</v>
+      </c>
+      <c r="F22" t="s">
+        <v>90</v>
+      </c>
+      <c r="G22" t="s">
+        <v>91</v>
+      </c>
+      <c r="H22" t="s">
         <v>92</v>
       </c>
-      <c r="F22" t="s">
-        <v>93</v>
-      </c>
-      <c r="G22" t="s">
-        <v>94</v>
-      </c>
-      <c r="H22" t="s">
-        <v>95</v>
-      </c>
       <c r="I22" s="24" t="s">
-        <v>248</v>
+        <v>191</v>
       </c>
       <c r="J22" t="s">
-        <v>247</v>
-      </c>
-      <c r="L22" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" ht="15.6">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="15.6">
       <c r="A23" s="2">
         <f>A22+3</f>
         <v>46090</v>
@@ -2375,28 +2190,25 @@
         <v>27</v>
       </c>
       <c r="E23" t="s">
-        <v>253</v>
+        <v>196</v>
       </c>
       <c r="F23" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="G23" t="s">
-        <v>249</v>
+        <v>192</v>
       </c>
       <c r="H23" t="s">
-        <v>250</v>
+        <v>193</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>252</v>
+        <v>195</v>
       </c>
       <c r="J23" t="s">
-        <v>251</v>
-      </c>
-      <c r="L23" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" ht="15.6">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="15.6">
       <c r="A24" s="2">
         <f>A23+2</f>
         <v>46092</v>
@@ -2412,25 +2224,25 @@
         <v>28</v>
       </c>
       <c r="E24" t="s">
-        <v>283</v>
+        <v>223</v>
       </c>
       <c r="F24" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="G24" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="H24" t="s">
-        <v>254</v>
+        <v>197</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>256</v>
+        <v>199</v>
       </c>
       <c r="J24" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" ht="15.6">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="15.6">
       <c r="A25" s="2">
         <f>A24+2</f>
         <v>46094</v>
@@ -2446,28 +2258,25 @@
         <v>29</v>
       </c>
       <c r="E25" t="s">
-        <v>284</v>
+        <v>224</v>
       </c>
       <c r="F25" t="s">
-        <v>262</v>
+        <v>204</v>
       </c>
       <c r="G25" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="H25" t="s">
-        <v>257</v>
+        <v>200</v>
       </c>
       <c r="I25" s="24" t="s">
-        <v>260</v>
+        <v>203</v>
       </c>
       <c r="J25" t="s">
-        <v>259</v>
-      </c>
-      <c r="L25" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" ht="15.6">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15.6">
       <c r="A26" s="2">
         <f>A25+3</f>
         <v>46097</v>
@@ -2483,31 +2292,25 @@
         <v>30</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F26" t="s">
-        <v>285</v>
+        <v>225</v>
       </c>
       <c r="G26" t="s">
-        <v>263</v>
+        <v>205</v>
       </c>
       <c r="H26" t="s">
-        <v>258</v>
+        <v>201</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>265</v>
+        <v>207</v>
       </c>
       <c r="J26" t="s">
-        <v>264</v>
-      </c>
-      <c r="L26" t="s">
-        <v>169</v>
-      </c>
-      <c r="M26" s="24" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" ht="15.6">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="15.6">
       <c r="A27" s="2">
         <f>A26+2</f>
         <v>46099</v>
@@ -2520,31 +2323,28 @@
         <v>Wed</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>268</v>
+        <v>209</v>
       </c>
       <c r="F27" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="G27" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H27" t="s">
-        <v>266</v>
+        <v>208</v>
       </c>
       <c r="I27" s="24" t="s">
-        <v>270</v>
+        <v>211</v>
       </c>
       <c r="J27" t="s">
-        <v>269</v>
-      </c>
-      <c r="L27" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" ht="15.6">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="15.6">
       <c r="A28" s="2">
         <f>A27+2</f>
         <v>46101</v>
@@ -2557,32 +2357,28 @@
         <v>Fri</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E28" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F28" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="G28" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H28" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>272</v>
+        <v>213</v>
       </c>
       <c r="J28" t="s">
-        <v>271</v>
-      </c>
-      <c r="L28" t="s">
-        <v>151</v>
-      </c>
-      <c r="M28" s="24"/>
-    </row>
-    <row r="29" spans="1:13" ht="15.6">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="15.6">
       <c r="A29" s="2">
         <f>A28+3</f>
         <v>46104</v>
@@ -2593,10 +2389,10 @@
         <v>Mon</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" ht="15.6">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="15.6">
       <c r="A30" s="2">
         <f>A29+2</f>
         <v>46106</v>
@@ -2607,10 +2403,10 @@
         <v>Wed</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" ht="15.6">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="15.6">
       <c r="A31" s="2">
         <f>A30+2</f>
         <v>46108</v>
@@ -2621,10 +2417,10 @@
         <v>Fri</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" ht="15.6">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="15.6">
       <c r="A32" s="2">
         <f>A31+3</f>
         <v>46111</v>
@@ -2637,28 +2433,28 @@
         <v>Mon</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E32" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="F32" t="s">
+        <v>107</v>
+      </c>
+      <c r="G32" t="s">
+        <v>227</v>
+      </c>
+      <c r="H32" t="s">
         <v>110</v>
       </c>
-      <c r="G32" t="s">
-        <v>287</v>
-      </c>
-      <c r="H32" t="s">
-        <v>113</v>
-      </c>
       <c r="I32" s="27" t="s">
-        <v>273</v>
+        <v>214</v>
       </c>
       <c r="J32" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" ht="15.6">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="15.6">
       <c r="A33" s="2">
         <f>A32+2</f>
         <v>46113</v>
@@ -2671,34 +2467,28 @@
         <v>Wed</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E33" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="F33" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="G33" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H33" t="s">
-        <v>282</v>
+        <v>222</v>
       </c>
       <c r="I33" s="27" t="s">
-        <v>275</v>
+        <v>216</v>
       </c>
       <c r="J33" t="s">
-        <v>276</v>
-      </c>
-      <c r="L33" t="s">
-        <v>177</v>
-      </c>
-      <c r="M33" s="24" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" ht="15.6">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="15.6">
       <c r="A34" s="2">
         <f>A33+2</f>
         <v>46115</v>
@@ -2711,32 +2501,28 @@
         <v>Fri</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E34" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F34" t="s">
-        <v>288</v>
+        <v>228</v>
       </c>
       <c r="G34" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="H34" t="s">
-        <v>280</v>
+        <v>220</v>
       </c>
       <c r="I34" s="27" t="s">
-        <v>277</v>
+        <v>218</v>
       </c>
       <c r="J34" t="s">
-        <v>278</v>
-      </c>
-      <c r="L34" t="s">
-        <v>279</v>
-      </c>
-      <c r="M34" s="24"/>
-    </row>
-    <row r="35" spans="1:13" ht="15.6">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="15.6">
       <c r="A35" s="2">
         <f>A34+3</f>
         <v>46118</v>
@@ -2749,34 +2535,28 @@
         <v>Mon</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E35" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F35" t="s">
-        <v>289</v>
+        <v>229</v>
       </c>
       <c r="G35" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H35" t="s">
-        <v>281</v>
+        <v>221</v>
       </c>
       <c r="I35" s="27" t="s">
-        <v>290</v>
+        <v>230</v>
       </c>
       <c r="J35" t="s">
-        <v>291</v>
-      </c>
-      <c r="L35" t="s">
-        <v>166</v>
-      </c>
-      <c r="M35" s="24" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" ht="15.6">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="15.6">
       <c r="A36" s="2">
         <f>A35+2</f>
         <v>46120</v>
@@ -2789,31 +2569,25 @@
         <v>Wed</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E36" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F36" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G36" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I36" s="27" t="s">
-        <v>292</v>
+        <v>232</v>
       </c>
       <c r="J36" t="s">
-        <v>293</v>
-      </c>
-      <c r="L36" t="s">
-        <v>171</v>
-      </c>
-      <c r="M36" s="24" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13" ht="16.2" thickBot="1">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="16.2" thickBot="1">
       <c r="A37" s="2">
         <f>A36+2</f>
         <v>46122</v>
@@ -2829,19 +2603,16 @@
         <v>2</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>0</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="L37" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13" ht="15.6">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="15.6">
       <c r="A38" s="2">
         <f>A37+3</f>
         <v>46125</v>
@@ -2857,26 +2628,23 @@
         <v>10</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="G38" s="9"/>
       <c r="H38" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I38" s="27" t="s">
-        <v>294</v>
+        <v>234</v>
       </c>
       <c r="J38" t="s">
-        <v>295</v>
-      </c>
-      <c r="L38" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13" ht="15.6">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="15.6">
       <c r="A39" s="2">
         <f>A38+2</f>
         <v>46127</v>
@@ -2892,19 +2660,16 @@
         <v>11</v>
       </c>
       <c r="H39" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I39" s="27" t="s">
-        <v>296</v>
+        <v>236</v>
       </c>
       <c r="J39" t="s">
-        <v>297</v>
-      </c>
-      <c r="L39" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="40" spans="1:13" ht="15.6">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="15.6">
       <c r="A40" s="2">
         <f>A39+2</f>
         <v>46129</v>
@@ -2917,19 +2682,22 @@
         <v>Fri</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G40" t="s">
-        <v>123</v>
+        <v>240</v>
       </c>
       <c r="H40" t="s">
-        <v>124</v>
-      </c>
-      <c r="L40" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13" ht="15.6">
+        <v>120</v>
+      </c>
+      <c r="I40" s="27" t="s">
+        <v>238</v>
+      </c>
+      <c r="J40" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="15.6">
       <c r="A41" s="2">
         <f>A40+3</f>
         <v>46132</v>
@@ -2942,19 +2710,16 @@
         <v>Mon</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="L41" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" ht="15.6">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="15.6">
       <c r="A42" s="2">
         <f>A41+2</f>
         <v>46134</v>
@@ -2967,22 +2732,28 @@
         <v>Wed</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="G42" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13" ht="15.6">
+        <v>245</v>
+      </c>
+      <c r="I42" s="27" t="s">
+        <v>243</v>
+      </c>
+      <c r="J42" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="15.6">
       <c r="A43" s="2">
         <f>A42+2</f>
         <v>46136</v>
@@ -2995,19 +2766,22 @@
         <v>Fri</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="G43" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="H43" t="s">
-        <v>129</v>
-      </c>
-      <c r="L43" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13" ht="15.6">
+        <v>241</v>
+      </c>
+      <c r="I43" s="27" t="s">
+        <v>246</v>
+      </c>
+      <c r="J43" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="15.6">
       <c r="A44" s="2">
         <f>A43+3</f>
         <v>46139</v>
@@ -3020,25 +2794,28 @@
         <v>Mon</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>38</v>
+        <v>251</v>
       </c>
       <c r="E44" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="G44" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="H44" t="s">
-        <v>128</v>
-      </c>
-      <c r="L44" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13" ht="15.6">
+        <v>242</v>
+      </c>
+      <c r="I44" s="27" t="s">
+        <v>248</v>
+      </c>
+      <c r="J44" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="15.6">
       <c r="A45" s="2">
         <f>A44+2</f>
         <v>46141</v>
@@ -3051,22 +2828,16 @@
         <v>Wed</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="L45" t="s">
-        <v>173</v>
-      </c>
-      <c r="M45" s="24" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="46" spans="1:13" ht="15.6">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="15.6">
       <c r="A46" s="14">
         <f>A45+2</f>
         <v>46143</v>
@@ -3085,14 +2856,11 @@
         <v>5</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="G46" s="9"/>
-      <c r="L46" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="47" spans="1:13" ht="15.6">
+    </row>
+    <row r="47" spans="1:10" ht="15.6">
       <c r="A47" s="2">
         <f>A46+3</f>
         <v>46146</v>
@@ -3105,20 +2873,17 @@
         <v>Mon</v>
       </c>
       <c r="D47" s="19" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E47" s="17" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="F47" s="18" t="s">
         <v>4</v>
       </c>
       <c r="G47" s="18"/>
-      <c r="L47" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="48" spans="1:13" ht="15.6">
+    </row>
+    <row r="48" spans="1:10" ht="15.6">
       <c r="A48" s="2">
         <f>A47+2</f>
         <v>46148</v>
@@ -3131,50 +2896,24 @@
         <v>Wed</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F48" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="50" spans="1:13">
-      <c r="L50" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="51" spans="1:13" ht="14.4">
+      <c r="G48" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" ht="14.4">
       <c r="A51" s="20"/>
       <c r="C51" s="21"/>
     </row>
-    <row r="52" spans="1:13" ht="14.4">
+    <row r="52" spans="1:3" ht="14.4">
       <c r="B52" s="21"/>
-      <c r="L52" t="s">
-        <v>182</v>
-      </c>
-      <c r="M52" s="24" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="55" spans="1:13">
-      <c r="L55" t="s">
-        <v>184</v>
-      </c>
-      <c r="M55" s="24" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="56" spans="1:13">
-      <c r="L56" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="60" spans="1:13">
-      <c r="L60" t="s">
-        <v>187</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3187,43 +2926,38 @@
     <hyperlink ref="I7" r:id="rId4" xr:uid="{510B6558-56CD-44A2-805A-B2C7949FF8EF}"/>
     <hyperlink ref="I8" r:id="rId5" xr:uid="{8F594743-93A9-4665-95A9-83C99405E5BD}"/>
     <hyperlink ref="I9" r:id="rId6" xr:uid="{22CA0FDC-A63D-456F-81DA-74E9A89775EE}"/>
-    <hyperlink ref="M9" r:id="rId7" xr:uid="{57DEC4EF-2D00-4E8D-9A77-300474F2F32A}"/>
-    <hyperlink ref="M10" r:id="rId8" xr:uid="{FEFB366C-46B5-4FCF-B20A-B66880D0CBB0}"/>
-    <hyperlink ref="I10" r:id="rId9" xr:uid="{81DBC2F5-857F-40BD-8614-8B92975625C0}"/>
-    <hyperlink ref="I11" r:id="rId10" xr:uid="{9DB554BE-F1E7-4A10-8857-6AD7EE61C4F9}"/>
-    <hyperlink ref="I12" r:id="rId11" xr:uid="{A0BE5509-76CC-47EB-8F87-CE802986609C}"/>
-    <hyperlink ref="I13" r:id="rId12" xr:uid="{17E1DBA7-1282-4B9C-AE93-3520A2CC1B70}"/>
-    <hyperlink ref="I14" r:id="rId13" xr:uid="{B2838FD0-63F6-4E7A-BA3A-876EF84E7420}"/>
-    <hyperlink ref="I15" r:id="rId14" xr:uid="{284CEF5E-CA76-42E6-ABDD-B2562CA15DD5}"/>
-    <hyperlink ref="I16" r:id="rId15" xr:uid="{740748D9-3731-4D44-90E6-D444B3DFFCDA}"/>
-    <hyperlink ref="I17" r:id="rId16" xr:uid="{66888497-A698-4D0D-A51C-3F6EF823B9DB}"/>
-    <hyperlink ref="I19" r:id="rId17" xr:uid="{4AC4DC58-D110-49BA-AE55-2D0EC7976090}"/>
-    <hyperlink ref="I20" r:id="rId18" xr:uid="{A4C4F584-67AC-4B2D-9137-C45F31F04441}"/>
-    <hyperlink ref="I21" r:id="rId19" xr:uid="{266AF027-98B3-4D9C-8AB8-C8B1B42BAD7B}"/>
-    <hyperlink ref="I22" r:id="rId20" xr:uid="{FEC1AA73-808D-4A29-9E5F-50B1A3E7721F}"/>
-    <hyperlink ref="I23" r:id="rId21" xr:uid="{8B44EAEB-E310-4371-8C4C-2F58A07E7C87}"/>
-    <hyperlink ref="I24" r:id="rId22" xr:uid="{3942BA65-4836-4C7A-95F8-6C4B19B38220}"/>
-    <hyperlink ref="I25" r:id="rId23" xr:uid="{EB0A94FC-1253-44E8-A838-2C52B3979496}"/>
-    <hyperlink ref="I26" r:id="rId24" xr:uid="{BFEB963A-7643-41BF-9C5D-4A5452BD9A9D}"/>
-    <hyperlink ref="I27" r:id="rId25" xr:uid="{F3195E4E-9BDD-4125-BBD6-A00170E588CA}"/>
-    <hyperlink ref="I28" r:id="rId26" xr:uid="{A7A55F02-5B29-4375-AB5F-BE0C0B59FFE1}"/>
-    <hyperlink ref="I32" r:id="rId27" xr:uid="{7BBB8307-26C1-4A6B-A11B-C046A9E889A3}"/>
-    <hyperlink ref="M33" r:id="rId28" xr:uid="{A99321CF-3833-4711-9272-617D4ADACDCC}"/>
-    <hyperlink ref="I33" r:id="rId29" xr:uid="{90B349C4-33E9-4C05-A37C-6D393BD1852A}"/>
-    <hyperlink ref="I34" r:id="rId30" xr:uid="{B4B1FB19-A42A-409A-B51B-5F25103A0C02}"/>
-    <hyperlink ref="M35" r:id="rId31" xr:uid="{4808DC9C-9621-475A-912C-A4349B18342E}"/>
-    <hyperlink ref="M26" r:id="rId32" xr:uid="{90B7AFE8-10E2-4E37-B21B-86B368CCBC7D}"/>
-    <hyperlink ref="M36" r:id="rId33" xr:uid="{5157CB41-CD23-479F-BF03-7DCA0601E8C4}"/>
-    <hyperlink ref="M45" r:id="rId34" xr:uid="{5AEB11BA-66D4-4B88-98BE-7B30D51D6CE2}"/>
-    <hyperlink ref="M52" r:id="rId35" xr:uid="{4FB78D27-EA2B-47A6-BF6B-7AA3C15BE02F}"/>
-    <hyperlink ref="M55" r:id="rId36" xr:uid="{C679864C-F1BF-40AB-9F12-9EE67A0B581C}"/>
-    <hyperlink ref="I35" r:id="rId37" xr:uid="{F2225EC5-E8B7-4715-A3DD-E8C926AFFBE9}"/>
-    <hyperlink ref="I36" r:id="rId38" xr:uid="{3191F546-109F-40A5-B0B8-48A63054C6DC}"/>
-    <hyperlink ref="I38" r:id="rId39" xr:uid="{7F488FF9-D4C9-4DFD-B169-AAE599D57542}"/>
-    <hyperlink ref="I39" r:id="rId40" xr:uid="{5A6D8735-3851-4571-89F6-B6E871265ABD}"/>
+    <hyperlink ref="I10" r:id="rId7" xr:uid="{81DBC2F5-857F-40BD-8614-8B92975625C0}"/>
+    <hyperlink ref="I11" r:id="rId8" xr:uid="{9DB554BE-F1E7-4A10-8857-6AD7EE61C4F9}"/>
+    <hyperlink ref="I12" r:id="rId9" xr:uid="{A0BE5509-76CC-47EB-8F87-CE802986609C}"/>
+    <hyperlink ref="I13" r:id="rId10" xr:uid="{17E1DBA7-1282-4B9C-AE93-3520A2CC1B70}"/>
+    <hyperlink ref="I14" r:id="rId11" xr:uid="{B2838FD0-63F6-4E7A-BA3A-876EF84E7420}"/>
+    <hyperlink ref="I15" r:id="rId12" xr:uid="{284CEF5E-CA76-42E6-ABDD-B2562CA15DD5}"/>
+    <hyperlink ref="I16" r:id="rId13" xr:uid="{740748D9-3731-4D44-90E6-D444B3DFFCDA}"/>
+    <hyperlink ref="I17" r:id="rId14" xr:uid="{66888497-A698-4D0D-A51C-3F6EF823B9DB}"/>
+    <hyperlink ref="I19" r:id="rId15" xr:uid="{4AC4DC58-D110-49BA-AE55-2D0EC7976090}"/>
+    <hyperlink ref="I20" r:id="rId16" xr:uid="{A4C4F584-67AC-4B2D-9137-C45F31F04441}"/>
+    <hyperlink ref="I21" r:id="rId17" xr:uid="{266AF027-98B3-4D9C-8AB8-C8B1B42BAD7B}"/>
+    <hyperlink ref="I22" r:id="rId18" xr:uid="{FEC1AA73-808D-4A29-9E5F-50B1A3E7721F}"/>
+    <hyperlink ref="I23" r:id="rId19" xr:uid="{8B44EAEB-E310-4371-8C4C-2F58A07E7C87}"/>
+    <hyperlink ref="I24" r:id="rId20" xr:uid="{3942BA65-4836-4C7A-95F8-6C4B19B38220}"/>
+    <hyperlink ref="I25" r:id="rId21" xr:uid="{EB0A94FC-1253-44E8-A838-2C52B3979496}"/>
+    <hyperlink ref="I26" r:id="rId22" xr:uid="{BFEB963A-7643-41BF-9C5D-4A5452BD9A9D}"/>
+    <hyperlink ref="I27" r:id="rId23" xr:uid="{F3195E4E-9BDD-4125-BBD6-A00170E588CA}"/>
+    <hyperlink ref="I28" r:id="rId24" xr:uid="{A7A55F02-5B29-4375-AB5F-BE0C0B59FFE1}"/>
+    <hyperlink ref="I32" r:id="rId25" xr:uid="{7BBB8307-26C1-4A6B-A11B-C046A9E889A3}"/>
+    <hyperlink ref="I33" r:id="rId26" xr:uid="{90B349C4-33E9-4C05-A37C-6D393BD1852A}"/>
+    <hyperlink ref="I34" r:id="rId27" xr:uid="{B4B1FB19-A42A-409A-B51B-5F25103A0C02}"/>
+    <hyperlink ref="I35" r:id="rId28" xr:uid="{F2225EC5-E8B7-4715-A3DD-E8C926AFFBE9}"/>
+    <hyperlink ref="I36" r:id="rId29" xr:uid="{3191F546-109F-40A5-B0B8-48A63054C6DC}"/>
+    <hyperlink ref="I38" r:id="rId30" xr:uid="{7F488FF9-D4C9-4DFD-B169-AAE599D57542}"/>
+    <hyperlink ref="I39" r:id="rId31" xr:uid="{5A6D8735-3851-4571-89F6-B6E871265ABD}"/>
+    <hyperlink ref="I40" r:id="rId32" xr:uid="{8F6B8108-DD3C-4289-A467-451C85593211}"/>
+    <hyperlink ref="I42" r:id="rId33" xr:uid="{3F17C56B-6F35-4988-8883-DE8FFF7E7326}"/>
+    <hyperlink ref="I43" r:id="rId34" xr:uid="{636CA437-ACF7-4C88-BDF0-0C4D90586AB3}"/>
+    <hyperlink ref="I44" r:id="rId35" xr:uid="{8D18B240-303A-4DA2-881B-EEB25165E0A3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="85" orientation="portrait" r:id="rId41"/>
+  <pageSetup scale="91" orientation="portrait" r:id="rId36"/>
   <ignoredErrors>
     <ignoredError sqref="A38 A41 A44 A47" formula="1"/>
   </ignoredErrors>

</xml_diff>